<commit_message>
Actualización de productos, usuarios y mejoras en el dashboard
</commit_message>
<xml_diff>
--- a/bd/registros.xlsx
+++ b/bd/registros.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1418,6 +1418,86 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Nuevo usuario registrado: tatiana</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2026-02-22 23:04:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026-02-22 23:11:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2026-02-23 12:49:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2026-02-23 13:29:17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
css, js, apardado admin principal
</commit_message>
<xml_diff>
--- a/bd/registros.xlsx
+++ b/bd/registros.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1418,6 +1418,206 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>elementorjj7@gmail.com</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Nuevo usuario registrado: jilmer</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2026-02-20 12:42:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026-02-20 12:51:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>hola@gmail.com</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Nuevo usuario registrado: jilmer</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2026-02-20 15:47:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>hola2@gmail.com</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Nuevo usuario registrado: Isabel</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2026-02-20 15:47:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>hola@gmail.com</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2026-02-20 15:47:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2026-02-20 16:01:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>2026-02-24 13:33:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2026-02-24 13:46:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2026-02-24 13:51:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2026-02-24 13:59:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
cambio admin usuario con apartado de descarga de tabla de registros
</commit_message>
<xml_diff>
--- a/bd/registros.xlsx
+++ b/bd/registros.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1078,6 +1078,26 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>74</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Actualizo usuario hola3@gmail.com (ID 5)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2026-02-25 15:32:33</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar archivos CSS y JS, actualizar app.py y archivos bd
</commit_message>
<xml_diff>
--- a/bd/registros.xlsx
+++ b/bd/registros.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1098,6 +1098,46 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2026-02-25 22:33:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>tatis@gmail.com</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Nuevo usuario registrado: Tatiana Rivera</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2026-02-25 22:35:53</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
sidebar y dashboard principal usuarios
</commit_message>
<xml_diff>
--- a/bd/registros.xlsx
+++ b/bd/registros.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1498,6 +1498,146 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>julio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2026-02-23 13:51:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>julio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2026-02-24 13:22:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>julio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>2026-02-24 13:26:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>julio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2026-02-24 15:00:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>julio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2026-02-24 16:55:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>julio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2026-02-25 12:54:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>2026-02-25 17:29:31</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
organizacion de carpetas css,js y los pedidos con el carrito
</commit_message>
<xml_diff>
--- a/bd/registros.xlsx
+++ b/bd/registros.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1138,6 +1138,566 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>tatis@gmail.com</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2026-02-25 23:15:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2026-02-25 23:16:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>tatis@gmail.com</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2026-02-25 23:17:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2026-02-26 22:52:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nuevo usuario registrado: Tatiana Rivera</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2026-02-26 22:54:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2026-02-26 22:57:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2026-02-26 23:02:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2026-02-26 23:05:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2026-02-26 23:20:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2026-02-27 12:31:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2026-02-27 12:53:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2026-02-27 12:55:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:03:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:03:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:41:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:48:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:49:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:51:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>julio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:52:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>julio@gmail.com</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:52:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:58:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2026-02-27 14:04:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2026-02-27 14:06:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2026-02-27 14:11:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>2026-02-27 14:11:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>2026-02-27 14:12:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>nico@gmail.com</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>2026-02-27 14:28:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>tr3303419@gmail.com</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Inicio de sesión exitoso</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2026-02-27 15:06:28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>